<commit_message>
Add interactive financial dashboard
</commit_message>
<xml_diff>
--- a/data/financial_data.xlsx
+++ b/data/financial_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mhxtyalo/Corporate-Intelligence-Lab/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06A96604-9488-E145-A2FE-1E57C6873E7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C0CFB8-5B17-0649-8A9A-D3D0DD292222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="16940" xr2:uid="{5782A1BD-547C-044C-B8BD-064DAC428F15}"/>
+    <workbookView xWindow="1060" yWindow="-15360" windowWidth="27320" windowHeight="15360" activeTab="1" xr2:uid="{5782A1BD-547C-044C-B8BD-064DAC428F15}"/>
   </bookViews>
   <sheets>
     <sheet name="Income_Statement" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="10">
   <si>
     <t>Company</t>
   </si>
@@ -447,7 +447,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C66A7A2-6672-F640-86F4-263C9E26BFEA}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.1640625" bestFit="1" customWidth="1"/>
@@ -472,13 +472,13 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="C2">
-        <v>23000</v>
+        <v>18000</v>
       </c>
       <c r="D2">
-        <v>1500</v>
+        <v>900</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -486,68 +486,194 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C3">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="D3">
-        <v>1800</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C4">
-        <v>80000</v>
+        <v>21500</v>
       </c>
       <c r="D4">
-        <v>14000</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C5">
-        <v>86000</v>
+        <v>23000</v>
       </c>
       <c r="D5">
-        <v>15000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C6">
-        <v>27000</v>
+        <v>25000</v>
       </c>
       <c r="D6">
-        <v>2800</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>2020</v>
+      </c>
+      <c r="C7">
+        <v>65000</v>
+      </c>
+      <c r="D7">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8">
+        <v>2021</v>
+      </c>
+      <c r="C8">
+        <v>70000</v>
+      </c>
+      <c r="D8">
+        <v>10500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9">
+        <v>2022</v>
+      </c>
+      <c r="C9">
+        <v>76000</v>
+      </c>
+      <c r="D9">
+        <v>12500</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10">
+        <v>2023</v>
+      </c>
+      <c r="C10">
+        <v>80000</v>
+      </c>
+      <c r="D10">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11">
+        <v>2024</v>
+      </c>
+      <c r="C11">
+        <v>86000</v>
+      </c>
+      <c r="D11">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="B12">
+        <v>2020</v>
+      </c>
+      <c r="C12">
+        <v>22000</v>
+      </c>
+      <c r="D12">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13">
+        <v>2021</v>
+      </c>
+      <c r="C13">
+        <v>23500</v>
+      </c>
+      <c r="D13">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14">
+        <v>2022</v>
+      </c>
+      <c r="C14">
+        <v>25000</v>
+      </c>
+      <c r="D14">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15">
+        <v>2023</v>
+      </c>
+      <c r="C15">
+        <v>27000</v>
+      </c>
+      <c r="D15">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16">
         <v>2024</v>
       </c>
-      <c r="C7">
+      <c r="C16">
         <v>29000</v>
       </c>
-      <c r="D7">
+      <c r="D16">
         <v>3200</v>
       </c>
     </row>
@@ -558,7 +684,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17B40A2F-EC10-0D46-87DA-7631A4D6F628}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -583,16 +709,16 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="C2">
-        <v>28000</v>
+        <v>22000</v>
       </c>
       <c r="D2">
-        <v>11000</v>
+        <v>8000</v>
       </c>
       <c r="E2">
-        <v>8500</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -600,83 +726,236 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C3">
-        <v>30000</v>
+        <v>24000</v>
       </c>
       <c r="D3">
-        <v>12000</v>
+        <v>9000</v>
       </c>
       <c r="E3">
-        <v>9000</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C4">
-        <v>130000</v>
+        <v>26000</v>
       </c>
       <c r="D4">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c r="E4">
-        <v>30000</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C5">
-        <v>140000</v>
+        <v>28000</v>
       </c>
       <c r="D5">
-        <v>55000</v>
+        <v>11000</v>
       </c>
       <c r="E5">
-        <v>32000</v>
+        <v>8500</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C6">
-        <v>62000</v>
+        <v>30000</v>
       </c>
       <c r="D6">
-        <v>19000</v>
+        <v>12000</v>
       </c>
       <c r="E6">
-        <v>17000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>2020</v>
+      </c>
+      <c r="C7">
+        <v>100000</v>
+      </c>
+      <c r="D7">
+        <v>40000</v>
+      </c>
+      <c r="E7">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8">
+        <v>2021</v>
+      </c>
+      <c r="C8">
+        <v>110000</v>
+      </c>
+      <c r="D8">
+        <v>43000</v>
+      </c>
+      <c r="E8">
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9">
+        <v>2022</v>
+      </c>
+      <c r="C9">
+        <v>120000</v>
+      </c>
+      <c r="D9">
+        <v>47000</v>
+      </c>
+      <c r="E9">
+        <v>29000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10">
+        <v>2023</v>
+      </c>
+      <c r="C10">
+        <v>130000</v>
+      </c>
+      <c r="D10">
+        <v>50000</v>
+      </c>
+      <c r="E10">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11">
+        <v>2024</v>
+      </c>
+      <c r="C11">
+        <v>140000</v>
+      </c>
+      <c r="D11">
+        <v>55000</v>
+      </c>
+      <c r="E11">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="B12">
+        <v>2020</v>
+      </c>
+      <c r="C12">
+        <v>50000</v>
+      </c>
+      <c r="D12">
+        <v>15000</v>
+      </c>
+      <c r="E12">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13">
+        <v>2021</v>
+      </c>
+      <c r="C13">
+        <v>54000</v>
+      </c>
+      <c r="D13">
+        <v>16500</v>
+      </c>
+      <c r="E13">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14">
+        <v>2022</v>
+      </c>
+      <c r="C14">
+        <v>58000</v>
+      </c>
+      <c r="D14">
+        <v>18000</v>
+      </c>
+      <c r="E14">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15">
+        <v>2023</v>
+      </c>
+      <c r="C15">
+        <v>62000</v>
+      </c>
+      <c r="D15">
+        <v>19000</v>
+      </c>
+      <c r="E15">
+        <v>17000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16">
         <v>2024</v>
       </c>
-      <c r="C7">
+      <c r="C16">
         <v>65000</v>
       </c>
-      <c r="D7">
+      <c r="D16">
         <v>21000</v>
       </c>
-      <c r="E7">
+      <c r="E16">
         <v>18000</v>
       </c>
     </row>

</xml_diff>